<commit_message>
QA docs: Day-in-Life D1 field-completeness rewrite + Bundle->Block terminology sweep
D1 (Setup Product) rewritten 6->8 cases after live-testing found the
original TC-D1-01 assumed a Slab Product already existed instead of
using Quick Material Setup Wizard, TC-D1-03 skipped the required PO
step entirely, TC-D1-04 treated a compute-only cost field as
directly editable, and TC-D1-06 wrongly claimed FG products get the
same Control Policy auto-fix as Slab/Block (split into a corrected
TC-D1-06b). Separately swept "Bundle" -> "Block" terminology across
both qa_data.py (19 spots, predates the 2026-08-16 UI rename) and
qa_data_day_in_life.py, including updating a stale BDL- sample code
to the current BLK-26-xxxx sequence prefix.
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-day-in-life.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-day-in-life.xlsx
@@ -489,14 +489,14 @@
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 39</t>
+          <t>Total test cases: 40</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 23 / 10 / 6</t>
+          <t>High / Medium / Low: 23 / 11 / 6</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -890,7 +890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -984,33 +984,41 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>สร้าง Material ครบทุกฟิลด์บังคับ</t>
+          <t>สร้าง Material ใหม่ผ่าน Quick Material Setup Wizard (สร้าง Slab + Block Product ให้อัตโนมัติ)</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ผู้ใช้มีสิทธิ์ EMG-O Internal Manager</t>
+          <t>ผู้ใช้มีสิทธิ์ EMG-O Internal Manager และมีสิทธิ์ Products/Create</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดเมนู Stone Material &gt; New
-2. กรอกฟิลด์บังคับให้ครบ
-3. กด Save</t>
+          <t>1. เปิดเมนู Configuration &gt; Quick Material Setup
+2. เลือก Setup Mode = "สร้าง Material ใหม่"
+3. กรอกทุกฟิลด์ตามคอลัมน์ข้อมูลตัวอย่าง (ติ๊ก "ขายทั้งก้อนได้ (Block Product)" ด้วย — จำเป็นสำหรับ TC-D1-03 ต่อไป)
+4. กด Confirm</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Name = "Test Marble 01"
+          <t>Setup Mode = "สร้าง Material ใหม่"
+Material Name = "Test Marble 01"
 Category = "Marble"
 Pricing Mode = "Serial (per-slab)"
-Costing Basis = "Area (Sq.Mt.)"
-Slab Product = เลือกสินค้าที่มีอยู่ เช่น "Carrara White Slab"</t>
+Origin Country = "Italy" (optional)
+Density (Ton/CBM) = 2.75 (optional — ใส่ไว้เพื่อใช้ต่อใน TC-D1-03)
+Slab Sales Price = 1,500
+Slab Cost = 1,000
+ขายทั้งก้อนได้ (Block Product) = ✔ ติ๊ก
+Block Sales Price = 18,000
+Block Cost = 15,000
+มี Finished Good = ไม่ติ๊ก (ทดสอบแยกใน TC-D1-06b)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บันทึกสำเร็จ ไม่มี error</t>
+          <t>สร้างสำเร็จ ไม่มี error — ระบบสร้าง 2 สินค้าให้อัตโนมัติ: (1) "Test Marble 01 - Slab" Tracking=Serial UoM=Unit และ (2) "Test Marble 01 - Block" Tracking=Lot UoM=m³ แล้วผูกทั้งคู่เข้ากับ Material ทันที (product_id + product_id_block) เปิด Material ดู Costing Basis จะเป็นค่าเริ่มต้น "Area (Sq.Mt.)" เสมอ (wizard ไม่มีฟิลด์นี้ให้กรอกโดยตรง)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1020,7 +1028,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>regression ของ TC-A1-01</t>
+          <t>regression ของ TC-A1-01 — ปรับ flow ให้ตรงกับ day-in-life.html สไลด์ 2 จริง (ใช้ wizard ไม่ใช่ฟอร์ม Material ตรงๆ ซึ่งต้องมี Slab Product อยู่ก่อนแล้วถึงจะเลือกได้ ไม่เหมาะกับ Material ใหม่เอี่ยม) — ⚠️ ต้องมีสิทธิ์ Products/Create ก่อน (group_emgo_internal_manager ยังไม่มี ณ 2026-08-27 ดู progress.md finding #1) ไม่งั้น wizard จะ error ตอนสร้าง Slab/Block Product นี้เป็น fixture หลัก ("Test Marble 01") ที่ TC-D1-02/03/03b/04 ใช้ต่อทั้งหมด</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1036,29 +1044,29 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Material มี Block/Lot อยู่แล้ว — พยายามเปลี่ยน Pricing Mode</t>
+          <t>Material มี Block อยู่แล้ว — พยายามเปลี่ยน Pricing Mode</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Material มี Block/Lot อย่างน้อย 1 รายการอยู่แล้ว</t>
+          <t>Material "Test Marble 01" มี Block อยู่แล้ว 1 ใบ (สร้างจาก TC-D1-03) — ถ้าทำ TC นี้ก่อน TC-D1-03 ให้สร้าง Block เปล่าๆ ของ Material นี้ไว้ก่อน 1 ใบพอ (Supplier/Warehouse/PO Line อะไรก็ได้ ขอแค่มี stone.bundle ผูกกับ Material นี้จริง)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Material นั้น
-2. พยายามเปลี่ยน Pricing Mode จาก Serial เป็น Lot (หรือกลับกัน)
+          <t>1. เปิด Material "Test Marble 01"
+2. เปลี่ยน Pricing Mode จาก "Serial (per-slab)" เป็น "Lot (aggregate, cheap stone)"
 3. กด Save</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>สลับค่า Pricing Mode ไปอีกฝั่งหนึ่ง</t>
+          <t>Pricing Mode: "Serial (per-slab)" → "Lot (aggregate, cheap stone)"</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ขึ้น error ภาษาไทยแจ้งว่า Pricing Mode ถูกล็อกแล้ว บันทึกไม่ผ่าน</t>
+          <t>บันทึกไม่ผ่าน ขึ้น error ข้อความเป๊ะๆ: "Pricing Mode ถูกล็อกแล้ว เพราะ Material นี้มี Block อยู่แล้ว — สลับระหว่าง Serial กับ Lot บน Material ที่มีสต็อกจริงจะทำให้สถานะสต็อกปนกันผิดพลาด"</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1084,30 +1092,44 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ตั้ง Density (ตัน/CBM) แล้วสร้าง Block ใหม่ — Weight (Ton) เติมให้อัตโนมัติ</t>
+          <t>สร้าง PO จริง + ยืนยัน แล้วสร้าง Block จาก PO นั้น — Weight (Ton) เติมให้อัตโนมัติจาก Density</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Material ตั้งค่า Density (ตัน/CBM) ไว้แล้ว เช่น Carrara White = 2.75</t>
+          <t>Material "Test Marble 01" มี Block Product แล้ว (จาก TC-D1-01) และตั้ง Density=2.75 ไว้แล้ว</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. สร้าง Block ใหม่ของ Material นี้
-2. กรอก Total CBM
-3. ดูช่อง Weight (Ton) โดยไม่ต้องพิมพ์เอง</t>
+          <t>1. เปิดเมนู Purchase &gt; Orders &gt; New
+2. เลือก Vendor = "Demo Quarry Co."
+3. กด "Add a line" เพิ่มบรรทัด: Product="Test Marble 01 - Block", Quantity=2.0, Unit Price=25,000 (Subtotal เติมอัตโนมัติ=50,000)
+4. กด "Confirm Order" (PO เปลี่ยนสถานะเป็น Purchase)
+5. เปิดเมนู Stone Slab &gt; Blocks &gt; New
+6. กรอก Material/Quality/Warehouse
+7. เลือก Purchase Order Line = บรรทัดของ PO ที่เพิ่งยืนยัน — สังเกต Supplier + Total CBM เติมให้อัตโนมัติทันที
+8. กรอก Thickness (M)
+9. ดูช่อง Weight (Ton) โดยไม่ต้องพิมพ์เอง แล้วกด Save</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Total CBM = 2.0
-Density = 2.75 ตัน/CBM</t>
+          <t>Vendor = "Demo Quarry Co."
+PO Line: Product="Test Marble 01 - Block", Quantity=2.0, Unit Price=25,000, Subtotal=50,000 (เติมอัตโนมัติ)
+—
+Material = "Test Marble 01"
+Quality = "First" (ค่าเริ่มต้น)
+Warehouse = "Empire Granite Warehouse (EG01)"
+Purchase Order Line = บรรทัด PO ที่เพิ่งยืนยัน
+Supplier = เติมอัตโนมัติ = "Demo Quarry Co."
+Total CBM = เติมอัตโนมัติ = 2.0
+Thickness (M) = 0.04</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Weight (Ton) เติมให้อัตโนมัติ = 5.5 (2.0 × 2.75) ทันทีที่กรอก/แก้ Total CBM</t>
+          <t>PO confirm สำเร็จ (state=Purchase) — ทันทีที่เลือก Purchase Order Line บนฟอร์ม Block: Supplier + Total CBM เติมให้อัตโนมัติ (2.0) แล้ว Weight (Ton) เติมต่อให้อัตโนมัติ = 5.5 (2.0 × 2.75) โดยไม่ต้องพิมพ์เอง บันทึกสำเร็จ (PO+Block นี้ใช้ fixture ต่อใน TC-D1-04 ด้วย)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1117,7 +1139,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>ฟีเจอร์ใหม่ 2026-08-25 ไม่เคยมี Test Case มาก่อน</t>
+          <t>ฟีเจอร์ใหม่ 2026-08-25 ไม่เคยมี Test Case มาก่อน — ⚠️ เพิ่ม field ที่ขาดไปจากเอกสารเดิม: Total CBM/Weight(Ton)/Purchase Order Line/Thickness(M) ทั้งหมด invisible บนฟอร์ม Block ถ้า Material ไม่มี Block Product (ดู stone_bundle_views.xml, group invisible="not material_has_block_product") และ 3 ใน 4 ฟิลด์นั้นเป็น required ทันทีที่ Material มี Block Product — ต้องมี PO จริง (confirm แล้ว) อยู่ก่อนถึงจะสร้าง Block ได้เลย ไม่ใช่กรอก Total CBM ลอยๆ ตามที่เอกสารเดิมเขียนไว้ เพิ่มขั้นตอนสร้าง PO เองในเคสนี้เลย (แทนที่จะสมมติไว้ใน precondition เฉยๆ) เพราะถ้าไม่มี PO จริงจะทดสอบขั้นต่อไปไม่ได้เลย</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -1138,13 +1160,14 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Block มี Weight (Ton) ที่เติมอัตโนมัติแล้วตาม TC-D1-03</t>
+          <t>Block จาก TC-D1-03 มี Weight (Ton) เติมอัตโนมัติแล้ว = 5.5</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. แก้ Weight (Ton) เป็นค่าจากตาชั่งจริงด้วยมือ
-2. กด Save โดยไม่แตะ Total CBM หรือ Material อีก</t>
+          <t>1. เปิด Block จาก TC-D1-03
+2. แก้ Weight (Ton) เป็นค่าจากตาชั่งจริงด้วยมือ
+3. กด Save โดยไม่แตะ Total CBM หรือ Material อีก</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1154,7 +1177,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ค่าที่กรอกมือถูกเก็บไว้ตามที่พิมพ์ ไม่ถูกคำนวณทับกลับเป็น 5.5</t>
+          <t>ค่าที่กรอกมือถูกเก็บไว้ตามที่พิมพ์ (5.65) ไม่ถูกคำนวณทับกลับเป็น 5.5</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1164,7 +1187,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>ฟีเจอร์ใหม่ 2026-08-25 — ตรวจว่าไม่ถูกเขียนทับจนกว่าจะแก้ CBM/Material อีกครั้ง</t>
+          <t>ฟีเจอร์ใหม่ 2026-08-25 — ตรวจว่าไม่ถูกเขียนทับจนกว่าจะแก้ Total CBM หรือ Material อีกครั้ง</t>
         </is>
       </c>
       <c r="I7" s="7" t="n"/>
@@ -1180,17 +1203,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Costing Basis = Area (ค่าเริ่มต้น) คำนวณ Cost ของแผ่นถูกต้อง</t>
+          <t>Costing Basis = Area (ค่าเริ่มต้น) คำนวณ Cost ของแผ่นถูกต้อง จากต้นทุนจริงของ PO</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Material ตั้ง Costing Basis = "Area (Sq.Mt.)" (ค่าเริ่มต้น)</t>
+          <t>Block จาก TC-D1-03 (PO Subtotal=50,000 ÷ Total CBM=2.0 = PO Cost/CBM 25,000 × Thickness 0.04m = PO Cost/Sq.Mt. 1,000; ไม่มี Container ผูก จึง Landed Cost/Sq.Mt.=0 → Cost/Sq.Mt. รวม = 1,000)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Bundle &gt; แท็บ Slabs &gt; เพิ่ม 1 แถว ระบุ Slab L / Slab H
+          <t>1. เปิด Block จาก TC-D1-03 &gt; แท็บ Slabs &gt; เพิ่ม 1 แถว ระบุ Slab L / Slab H
 2. ตรวจ Cost ของแผ่นที่ได้</t>
         </is>
       </c>
@@ -1198,12 +1221,12 @@
         <is>
           <t>Slab L (M) = 2.0
 Slab H (M) = 1.5
-Cost / Sq.Mt. ของ Bundle = 1,000</t>
+(Cost/Sq.Mt. ของ Block = 1,000 — คำนวณอัตโนมัติจาก PO ไม่ต้องกรอกเอง ดู precondition)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Cost = 3,000 (2.0 × 1.5 × 1,000)</t>
+          <t>Cost = 3,000 (Slab Sq.Mt. 3.0 × Cost/Sq.Mt. 1,000)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1213,7 +1236,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>regression ของ TC-A3-04</t>
+          <t>regression ของ TC-A3-04 — ⚠️ แก้จากเอกสารเดิม: cost_sqmt/po_cost_sqmt เป็น compute field (ADR-005, 2026-08-02) ไม่ใช่ช่องให้พิมพ์ตรงๆ อย่างที่เอกสารเดิมสมมติ ต้องมาจากสูตร po_cost_cbm(=PO Subtotal÷Total CBM) × Thickness(M) จริง — ปรับ field ให้ครบเพื่อให้ได้ Cost/Sq.Mt.=1,000 เท่าเดิม</t>
         </is>
       </c>
       <c r="I8" s="7" t="n"/>
@@ -1229,29 +1252,34 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>ผูก Slab Product ที่ Control Policy เดิมเป็น "Received quantities"</t>
+          <t>สร้าง Material ใหม่ผ่านฟอร์ม Materials ตรงๆ (ไม่ใช่ Wizard) โดยผูก Slab Product ที่มีอยู่แล้ว — Control Policy เดิมเป็น "Received quantities"</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>มีสินค้าที่ตั้ง Control Policy (แท็บ Purchase) = "Received quantities" อยู่ก่อน</t>
+          <t>มีสินค้า "Test Onyx Slab (Pre-existing)" สร้างไว้ล่วงหน้าแล้ว (Sales &gt; Products &gt; New: Product Type=Goods, Track Inventory=✔, Tracking=By Unique Serial Number, UoM=Unit, Control Policy แท็บ Purchase = "Received quantities")</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>1. สร้าง Material ใหม่ ผูก Slab Product เป็นสินค้านั้น
-2. กด Save
-3. เปิดสินค้านั้นดูแท็บ Purchase อีกครั้ง</t>
+          <t>1. เปิดเมนู Configuration &gt; Materials &gt; New
+2. กรอก Material Name/Category/Pricing Mode
+3. ผูก Slab Product = "Test Onyx Slab (Pre-existing)"
+4. กด Save
+5. เปิดสินค้านั้นอีกครั้งดูแท็บ Purchase</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Slab Product = สินค้าที่ Control Policy เดิม = "Received quantities"</t>
+          <t>Material Name = "Test Onyx 01"
+Category = "Other"
+Pricing Mode = "Serial (per-slab)"
+Slab Product = "Test Onyx Slab (Pre-existing)" (Control Policy เดิม = "Received quantities")</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Control Policy ของสินค้าถูกเปลี่ยนเป็น "Ordered quantities" ให้อัตโนมัติ</t>
+          <t>บันทึกสำเร็จ ไม่มี error — เปิดสินค้า "Test Onyx Slab (Pre-existing)" อีกครั้ง Control Policy (แท็บ Purchase) ถูกเปลี่ยนเป็น "Ordered quantities" ให้อัตโนมัติ</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1261,7 +1289,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>regression ของ TC-A4-01 — กันบิลได้ยอด 0 เพราะไม่เคยยืนยันใบรับสินค้าจริง</t>
+          <t>regression ของ TC-A4-01 — กันบิลได้ยอด 0 เพราะไม่เคยยืนยันใบรับสินค้าจริง — ⚠️ ต้องใช้เมนู Configuration &gt; Materials &gt; New ตรงๆ เท่านั้น ห้ามใช้ Quick Material Setup Wizard เพราะ wizard สร้าง Slab Product ใหม่ให้เสมอ ไม่รองรับการเลือกสินค้าที่มีอยู่แล้ว — fixture นี้ ("Test Onyx 01") แยกจาก "Test Marble 01" เพื่อไม่ให้ชนกับ Block Product ที่ D1-01 สร้างให้ไปแล้ว</t>
         </is>
       </c>
       <c r="I9" s="7" t="n"/>
@@ -1277,30 +1305,30 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>ผูก Block Product + Finished Good Product ให้ Material เดียวกัน</t>
+          <t>ผูก Block Product ที่มีอยู่แล้วให้ Material เดียวกัน (Fixture B) — Control Policy เดิมเป็น "Received quantities"</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Material มีอยู่แล้ว (Slab Product ผูกครบ)</t>
+          <t>Material "Test Onyx 01" จาก TC-D1-05 มีอยู่แล้ว (Slab Product ผูกครบ) และมีสินค้าอีกตัว "Test Onyx Block (Pre-existing)" ตั้ง Control Policy เดิม = "Received quantities" ไว้ล่วงหน้า</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Material
-2. ผูก Block Product เป็นสินค้าที่ Control Policy เดิม = "Received quantities"
-3. ผูก Finished Good Product เป็นสินค้าอีกตัวที่ Control Policy เดิมเหมือนกัน
-4. กด Save แล้วเปิดทั้งสองสินค้าดูแท็บ Purchase</t>
+          <t>1. เปิด Material "Test Onyx 01"
+2. ผูก Block Product = "Test Onyx Block (Pre-existing)"
+3. กด Save
+4. เปิดสินค้านั้นดูแท็บ Purchase</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Block Product / Finished Good Product = สินค้าที่ Control Policy เดิม = "Received quantities" ทั้งคู่</t>
+          <t>Block Product = "Test Onyx Block (Pre-existing)" (Control Policy เดิม = "Received quantities")</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Control Policy ของทั้งสองสินค้าถูกเปลี่ยนเป็น "Ordered quantities" เหมือนกัน</t>
+          <t>Control Policy ของ Block Product ถูกเปลี่ยนเป็น "Ordered quantities" ให้อัตโนมัติ (เหมือน Slab Product ใน TC-D1-05)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1310,13 +1338,63 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>regression เบา ของ TC-A4-02/04 — Block/FG เป็นตัวเลือกเสริม หลักการเดียวกับ Slab Product</t>
+          <t>regression เบา ของ TC-A4-02 — Block Product เป็นตัวเลือกเสริม หลักการเดียวกับ Slab Product (TC-D1-05) — ⚠️ แยก FG ออกเป็น TC-D1-06b ต่างหากแล้ว เพราะพฤติกรรมจริงต่างกัน ไม่ใช่กรณีเดียวกับ Slab/Block</t>
         </is>
       </c>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>TC-D1-06b</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>ผูก Finished Good Product (stone_is_fg) เข้ากับ Material — Control Policy ไม่ถูกแก้ให้อัตโนมัติ (ต่างจาก Slab/Block)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Material "Test Onyx 01" มีอยู่แล้ว และมีสินค้าอีกตัว "Test Onyx FG (Pre-existing)" ตั้ง Control Policy เดิม = "Received quantities" ไว้ล่วงหน้า (ยังไม่ติ๊ก stone_is_fg)</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดสินค้า "Test Onyx FG (Pre-existing)" (Sales &gt; Products)
+2. ติ๊ก "Is Stone FG Product"
+3. เลือก "FG Raw Material" = Material "Test Onyx 01"
+4. กด Save
+5. ดูแท็บ Purchase อีกครั้ง</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>FG Raw Material = "Test Onyx 01"</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Save สำเร็จ — Tracking ถูกบังคับเป็น "By Lots" และ Track Inventory ติดอัตโนมัติ แต่ Control Policy (แท็บ Purchase) ยังเป็น "Received quantities" เดิม ไม่ถูกเปลี่ยน — ต่างจาก Slab/Block ที่ auto-fix ให้ (ความเสี่ยง: ถ้า FG ตัวนี้เคยซื้อขายจริงและไม่เคย confirm ใบรับสินค้า จะออกบิลได้ยอด 0 — ยังไม่ถูกแก้ในโค้ด)</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>⚠️ เอกสารเดิมเข้าใจผิดว่า FG Product ถูก auto-fix Control Policy เหมือน Slab/Block — เช็คโค้ดจริงแล้ว stone_material.py._ensure_purchase_method() ครอบคลุมเฉพาะ product_id/product_id_block เท่านั้น product_template.py._ensure_stone_fg_tracking() (ทำงานตอนติ๊ก stone_is_fg) จัดการแค่ Tracking/Track Inventory ไม่แตะ Control Policy เลย — แก้ expected result ให้ตรงกับโค้ดจริง ไม่ใช่การเปลี่ยนพฤติกรรม</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
+      <c r="L11" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2590,7 +2668,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Bundle ยังไม่มี SO ผูก แต่ต้องการตัดเข้าสต็อกไว้ล่วงหน้า</t>
+          <t>Block ยังไม่มี SO ผูก แต่ต้องการตัดเข้าสต็อกไว้ล่วงหน้า</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">

</xml_diff>